<commit_message>
chore: reconcile external link handoff state
</commit_message>
<xml_diff>
--- a/outputs/external-link-handoff-2026-08-02/外链提交交接表.xlsx
+++ b/outputs/external-link-handoff-2026-08-02/外链提交交接表.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="免费提交队列" sheetId="1" r:id="Ra275145d8cfa4f28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日提交记录" sheetId="2" r:id="R11ac173bc1284339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阻塞与排除" sheetId="3" r:id="R001624ee059c47fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI交接说明" sheetId="4" r:id="Reedb04a4ca644816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="免费提交队列" sheetId="1" r:id="R77013577b3a44db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日提交记录" sheetId="2" r:id="Ra53d91986f3d4af9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阻塞与排除" sheetId="3" r:id="Red0d450c0f514c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI交接说明" sheetId="4" r:id="R07119a4b31be4319"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -112,7 +112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +215,10 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -226,7 +230,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -236,7 +240,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -247,14 +251,14 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -264,7 +268,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -275,7 +279,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -311,7 +315,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodaySubmissionLog" displayName="TodaySubmissionLog" ref="A4:G16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodaySubmissionLog" displayName="TodaySubmissionLog" ref="A4:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="平台"/>
     <x:tableColumn id="2" name="链接 / 回执"/>
@@ -588,8 +592,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="10" t="n">
-        <x:f>COUNTIF(F6:F200,"待提交")</x:f>
-        <x:v>38</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B4" s="10"/>
       <x:c r="C4" s="10" t="n">
@@ -598,8 +601,7 @@
       </x:c>
       <x:c r="D4" s="10"/>
       <x:c r="E4" s="10" t="n">
-        <x:f>COUNTIF(F6:F200,"已提交/待审核")+COUNTIF(F6:F200,"已提交/排队")+COUNTIF(F6:F200,"已提交/已排期")</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F4" s="10"/>
       <x:c r="G4" s="10" t="n">
@@ -1033,7 +1035,7 @@
       <x:c r="F16" s="25" t="str">
         <x:v>待提交</x:v>
       </x:c>
-      <x:c r="G16" s="31" t="str"/>
+      <x:c r="G16" s="31"/>
       <x:c r="H16" s="25" t="str">
         <x:v>待验证</x:v>
       </x:c>
@@ -1052,7 +1054,7 @@
     </x:row>
     <x:row r="17" ht="44" customHeight="1">
       <x:c r="A17" s="28" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B17" s="25" t="str">
         <x:v>SideProjectors</x:v>
@@ -1061,26 +1063,28 @@
         <x:v>sideprojectors.com</x:v>
       </x:c>
       <x:c r="D17" s="25" t="str">
-        <x:v>来源标注免费（待复核）</x:v>
+        <x:v>已确认免费</x:v>
       </x:c>
       <x:c r="E17" s="25" t="str">
         <x:v>https://www.sideprojectors.com/submit</x:v>
       </x:c>
       <x:c r="F17" s="25" t="str">
-        <x:v>待提交</x:v>
-      </x:c>
-      <x:c r="G17" s="31" t="str"/>
+        <x:v>已提交/待审核</x:v>
+      </x:c>
+      <x:c r="G17" s="31" t="n">
+        <x:v>46236</x:v>
+      </x:c>
       <x:c r="H17" s="25" t="str">
-        <x:v>待验证</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="I17" s="25" t="str">
-        <x:v>按站点要求；上传后核对 files/预览</x:v>
+        <x:v>已完成真实表单提交</x:v>
       </x:c>
       <x:c r="J17" s="25" t="str">
-        <x:v>您的项目正在审核中，通常需要 2-3 个工作日才能获批。当您的项目获批时，我们将通过电子邮件通知您。</x:v>
+        <x:v>项目 ID 87446；确认页显示审核中，通常需要 2-3 个工作日</x:v>
       </x:c>
       <x:c r="K17" s="25" t="str">
-        <x:v>打开入口，先复核免费路线再填表</x:v>
+        <x:v>跳过，不重复提交；等待审核邮件</x:v>
       </x:c>
       <x:c r="L17" s="25" t="str">
         <x:v>https://www.sideprojectors.com/submit</x:v>
@@ -1664,7 +1668,7 @@
     </x:row>
     <x:row r="34" ht="44" customHeight="1">
       <x:c r="A34" s="28" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B34" s="25" t="str">
         <x:v>PitchWall</x:v>
@@ -1673,26 +1677,28 @@
         <x:v>pitchwall.co</x:v>
       </x:c>
       <x:c r="D34" s="25" t="str">
-        <x:v>来源标注免费（待复核）</x:v>
+        <x:v>已确认免费</x:v>
       </x:c>
       <x:c r="E34" s="25" t="str">
         <x:v>https://pitchwall.co/</x:v>
       </x:c>
       <x:c r="F34" s="25" t="str">
-        <x:v>待提交</x:v>
-      </x:c>
-      <x:c r="G34" s="31" t="str"/>
+        <x:v>已提交/待审核</x:v>
+      </x:c>
+      <x:c r="G34" s="31" t="n">
+        <x:v>46236</x:v>
+      </x:c>
       <x:c r="H34" s="25" t="str">
-        <x:v>待验证</x:v>
+        <x:v>无</x:v>
       </x:c>
       <x:c r="I34" s="25" t="str">
-        <x:v>按站点要求；上传后核对 files/预览</x:v>
+        <x:v>Logo、主图和截图已上传并核对预览</x:v>
       </x:c>
       <x:c r="J34" s="25" t="str">
-        <x:v>PitchWall; Free; DR 64; product/startup launch listing.</x:v>
+        <x:v>账户显示 Product Status: Under Review；免费发布预计超过 30 天</x:v>
       </x:c>
       <x:c r="K34" s="25" t="str">
-        <x:v>打开入口，先复核免费路线再填表</x:v>
+        <x:v>跳过，不重复提交；等待发布</x:v>
       </x:c>
       <x:c r="L34" s="25" t="str">
         <x:v>https://pitchwall.co/</x:v>
@@ -2482,7 +2488,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5df53f6a46cd417f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26510e2ca45c495f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2809,6 +2815,52 @@
         <x:v>人工注册后恢复</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="44" customHeight="1">
+      <x:c r="A17" s="45" t="str">
+        <x:v>SideProjectors</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="str">
+        <x:v>https://www.sideprojectors.com/submit</x:v>
+      </x:c>
+      <x:c r="C17" s="45" t="str">
+        <x:v>成功</x:v>
+      </x:c>
+      <x:c r="D17" s="45" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+      <x:c r="F17" s="45" t="str">
+        <x:v>项目 ID 87446；确认页显示正在审核，通常需要 2-3 个工作日</x:v>
+      </x:c>
+      <x:c r="G17" s="45" t="str">
+        <x:v>等待审核邮件；不要重复提交</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="44" customHeight="1">
+      <x:c r="A18" s="45" t="str">
+        <x:v>PitchWall</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="str">
+        <x:v>https://pitchwall.co/</x:v>
+      </x:c>
+      <x:c r="C18" s="45" t="str">
+        <x:v>成功</x:v>
+      </x:c>
+      <x:c r="D18" s="45" t="str">
+        <x:v>agent</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="n">
+        <x:v>46236</x:v>
+      </x:c>
+      <x:c r="F18" s="45" t="str">
+        <x:v>账户显示 Product Status: Under Review</x:v>
+      </x:c>
+      <x:c r="G18" s="45" t="str">
+        <x:v>免费方案预计超过 30 天发布；不要重复提交</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -2821,7 +2873,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196091a3d94345eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d7f598884e84ac2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3042,7 +3094,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra180564c39174631"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b65c469f1bb4b59"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>